<commit_message>
fix: get renaksi data
</commit_message>
<xml_diff>
--- a/evaluasi-kinerja-summary-2026-TW1.xlsx
+++ b/evaluasi-kinerja-summary-2026-TW1.xlsx
@@ -436,25 +436,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B2" t="str">
-        <v>222663</v>
+        <v>222659</v>
       </c>
       <c r="C2" t="str">
-        <v>ZAINAL NUR ROKIB</v>
+        <v>RIZKI PORMAN SIDABUTAR</v>
       </c>
       <c r="D2" t="str">
         <v>STAF</v>
       </c>
       <c r="E2" t="str">
-        <v>SDN JOHAR BARU 17</v>
+        <v>SDN JOHAR BARU 07 PAGI</v>
       </c>
       <c r="F2" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G2" t="str">
-        <v>Belum Ada</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H2" t="str">
-        <v>3783748</v>
+        <v>3785646</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -468,25 +468,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B3" t="str">
-        <v>222212</v>
+        <v>222661</v>
       </c>
       <c r="C3" t="str">
-        <v>ERICK LAUSHEN</v>
+        <v>IHZA MAHENDRA</v>
       </c>
       <c r="D3" t="str">
         <v>STAF</v>
       </c>
       <c r="E3" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SDN JOHAR BARU 10</v>
       </c>
       <c r="F3" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G3" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H3" t="str">
-        <v>3764322</v>
+        <v>3763494</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -500,25 +500,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B4" t="str">
-        <v>222219</v>
+        <v>186620</v>
       </c>
       <c r="C4" t="str">
-        <v>ISNAENI NURFALAH</v>
+        <v>ENDANG ERWIN</v>
       </c>
       <c r="D4" t="str">
-        <v>STAF</v>
+        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
       </c>
       <c r="E4" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SMPN 118 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F4" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G4" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H4" t="str">
-        <v>3764541</v>
+        <v>3767642</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -532,25 +532,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B5" t="str">
-        <v>222206</v>
+        <v>222645</v>
       </c>
       <c r="C5" t="str">
-        <v>FARIZ SEPTIAN</v>
+        <v>MEGANANDA DWI FITRIYANI</v>
       </c>
       <c r="D5" t="str">
         <v>STAF</v>
       </c>
       <c r="E5" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SDN HARAPAN MULIA 01</v>
       </c>
       <c r="F5" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G5" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H5" t="str">
-        <v>3771045</v>
+        <v>3783067</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -564,25 +564,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B6" t="str">
-        <v>222218</v>
+        <v>222666</v>
       </c>
       <c r="C6" t="str">
-        <v>NIRWANA PRATIWI</v>
+        <v>SYAFRIZAL</v>
       </c>
       <c r="D6" t="str">
         <v>STAF</v>
       </c>
       <c r="E6" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SDN TANAH TINGGI 05</v>
       </c>
       <c r="F6" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G6" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H6" t="str">
-        <v>3785348</v>
+        <v>3769614</v>
       </c>
       <c r="I6">
         <v>1</v>
@@ -596,25 +596,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B7" t="str">
-        <v>182677</v>
+        <v>222210</v>
       </c>
       <c r="C7" t="str">
-        <v>R.M. NURUL ZAMAN</v>
+        <v>MUHAMAD ALFARISI</v>
       </c>
       <c r="D7" t="str">
-        <v>KEPALA SUBBAGIAN TATA USAHA</v>
+        <v>STAF</v>
       </c>
       <c r="E7" t="str">
-        <v>SMAN 27 KECAMATAN JOHAR BARU</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F7" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G7" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H7" t="str">
-        <v>3772507</v>
+        <v>3770283</v>
       </c>
       <c r="I7">
         <v>1</v>
@@ -628,25 +628,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B8" t="str">
-        <v>189725</v>
+        <v>222211</v>
       </c>
       <c r="C8" t="str">
-        <v>HERYADI</v>
+        <v>PAMUNGKAS GUMILANG AJI</v>
       </c>
       <c r="D8" t="str">
-        <v>STAF PELAYANAN TINGKAT TERAMPIL</v>
+        <v>STAF</v>
       </c>
       <c r="E8" t="str">
-        <v>SDN PASEBAN 15 PAGI</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F8" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G8" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H8" t="str">
-        <v>3762438</v>
+        <v>3761250</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -660,25 +660,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B9" t="str">
-        <v>222649</v>
+        <v>222224</v>
       </c>
       <c r="C9" t="str">
-        <v>AHMAD SUPRIYANTO</v>
+        <v>IHSAN MAULANA ILMI</v>
       </c>
       <c r="D9" t="str">
         <v>STAF</v>
       </c>
       <c r="E9" t="str">
-        <v>SDN SUMUR BATU 14</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F9" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G9" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H9" t="str">
-        <v>3775544</v>
+        <v>3762076</v>
       </c>
       <c r="I9">
         <v>1</v>
@@ -692,25 +692,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B10" t="str">
-        <v>222216</v>
+        <v>197054</v>
       </c>
       <c r="C10" t="str">
-        <v>DESI RATNA SARI MARIA</v>
+        <v>ANDRIE GUSTYAJI</v>
       </c>
       <c r="D10" t="str">
-        <v>STAF</v>
+        <v>STAF TEKNIS TINGKAT AHLI</v>
       </c>
       <c r="E10" t="str">
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F10" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G10" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H10" t="str">
-        <v>3761422</v>
+        <v>3767464</v>
       </c>
       <c r="I10">
         <v>1</v>
@@ -724,10 +724,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B11" t="str">
-        <v>222221</v>
+        <v>222219</v>
       </c>
       <c r="C11" t="str">
-        <v>TASKIA ROROINTAN SUGYANTI</v>
+        <v>ISNAENI NURFALAH</v>
       </c>
       <c r="D11" t="str">
         <v>STAF</v>
@@ -736,13 +736,13 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F11" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G11" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H11" t="str">
-        <v>3775540</v>
+        <v>3764541</v>
       </c>
       <c r="I11">
         <v>1</v>
@@ -756,25 +756,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B12" t="str">
-        <v>163673</v>
+        <v>121949</v>
       </c>
       <c r="C12" t="str">
-        <v>SEMIATI</v>
+        <v>RIA SCORPIONI</v>
       </c>
       <c r="D12" t="str">
-        <v>KEPALA SUBBAGIAN TATA USAHA</v>
+        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E12" t="str">
-        <v>SMAN 30 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SMPN 79 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F12" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G12" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H12" t="str">
-        <v>3765532</v>
+        <v>3784557</v>
       </c>
       <c r="I12">
         <v>1</v>
@@ -788,10 +788,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B13" t="str">
-        <v>186567</v>
+        <v>135533</v>
       </c>
       <c r="C13" t="str">
-        <v>DAHIYAT</v>
+        <v>ENDANG RAHAYU NINGSIH</v>
       </c>
       <c r="D13" t="str">
         <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
@@ -800,13 +800,13 @@
         <v>SMPN 137 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F13" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G13" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H13" t="str">
-        <v>3784901</v>
+        <v>3767188</v>
       </c>
       <c r="I13">
         <v>1</v>
@@ -820,25 +820,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B14" t="str">
-        <v>165394</v>
+        <v>186021</v>
       </c>
       <c r="C14" t="str">
-        <v>ERWIN VICTOR PARULIAN</v>
+        <v>EDY SARWOKO</v>
       </c>
       <c r="D14" t="str">
         <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E14" t="str">
-        <v>SMKN 39 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SMKN 31 KECAMATAN JOHAR BARU</v>
       </c>
       <c r="F14" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G14" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H14" t="str">
-        <v>3770291</v>
+        <v>3767087</v>
       </c>
       <c r="I14">
         <v>1</v>
@@ -852,25 +852,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B15" t="str">
-        <v>141357</v>
+        <v>188772</v>
       </c>
       <c r="C15" t="str">
-        <v>HERI BUDI PRASETYA</v>
+        <v>SUTARNO</v>
       </c>
       <c r="D15" t="str">
-        <v>KEPALA SUBBAGIAN TATA USAHA</v>
+        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E15" t="str">
-        <v>SMAN 68 KECAMATAN SENEN</v>
+        <v>SMPN 28 KECAMATAN JOHAR BARU</v>
       </c>
       <c r="F15" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G15" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H15" t="str">
-        <v>3771889</v>
+        <v>3764714</v>
       </c>
       <c r="I15">
         <v>1</v>
@@ -884,25 +884,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B16" t="str">
-        <v>173346</v>
+        <v>137905</v>
       </c>
       <c r="C16" t="str">
-        <v>RISKY AMELIA</v>
+        <v>MELIA</v>
       </c>
       <c r="D16" t="str">
         <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E16" t="str">
-        <v>SMPN 47 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SMPN 76 KECAMATAN JOHAR BARU</v>
       </c>
       <c r="F16" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G16" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H16" t="str">
-        <v>3767707</v>
+        <v>3764712</v>
       </c>
       <c r="I16">
         <v>1</v>
@@ -916,25 +916,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B17" t="str">
-        <v>222657</v>
+        <v>182690</v>
       </c>
       <c r="C17" t="str">
-        <v>MUHAMMAD NADHIRSYAH INDRA</v>
+        <v>SALYA</v>
       </c>
       <c r="D17" t="str">
-        <v>STAF</v>
+        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E17" t="str">
-        <v>SDN JOHAR BARU 03</v>
+        <v>SMPN 71 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F17" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G17" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H17" t="str">
-        <v>3779978</v>
+        <v>3766145</v>
       </c>
       <c r="I17">
         <v>1</v>
@@ -948,25 +948,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B18" t="str">
-        <v>171293</v>
+        <v>222646</v>
       </c>
       <c r="C18" t="str">
-        <v>DEVIA ROSA</v>
+        <v>RETNO WULANDARI</v>
       </c>
       <c r="D18" t="str">
-        <v>KEPALA SUBBAGIAN TATA USAHA</v>
+        <v>STAF</v>
       </c>
       <c r="E18" t="str">
-        <v>SMAN 5 KECAMATAN KEMAYORAN</v>
+        <v>SDN HARAPAN MULIA 03</v>
       </c>
       <c r="F18" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G18" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H18" t="str">
-        <v>3762691</v>
+        <v>3765436</v>
       </c>
       <c r="I18">
         <v>1</v>
@@ -980,25 +980,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B19" t="str">
-        <v>222661</v>
+        <v>171594</v>
       </c>
       <c r="C19" t="str">
-        <v>IHZA MAHENDRA</v>
+        <v>SAFITRI HARUN</v>
       </c>
       <c r="D19" t="str">
-        <v>STAF</v>
+        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E19" t="str">
-        <v>SDN JOHAR BARU 10</v>
+        <v>SMPN 118 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F19" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G19" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H19" t="str">
-        <v>3763494</v>
+        <v>3763657</v>
       </c>
       <c r="I19">
         <v>1</v>
@@ -1012,10 +1012,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B20" t="str">
-        <v>222211</v>
+        <v>222207</v>
       </c>
       <c r="C20" t="str">
-        <v>PAMUNGKAS GUMILANG AJI</v>
+        <v>YAN AJIE PRASETIA</v>
       </c>
       <c r="D20" t="str">
         <v>STAF</v>
@@ -1024,13 +1024,13 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F20" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G20" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H20" t="str">
-        <v>3761250</v>
+        <v>3762888</v>
       </c>
       <c r="I20">
         <v>1</v>
@@ -1044,25 +1044,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B21" t="str">
-        <v>222208</v>
+        <v>222656</v>
       </c>
       <c r="C21" t="str">
-        <v>KUNTI DEWI AFIFA</v>
+        <v>HANDY WICAKSONO</v>
       </c>
       <c r="D21" t="str">
         <v>STAF</v>
       </c>
       <c r="E21" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SDN JOHAR BARU 01 PAGI</v>
       </c>
       <c r="F21" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G21" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H21" t="str">
-        <v>3773218</v>
+        <v>3783616</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -1076,25 +1076,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B22" t="str">
-        <v>185754</v>
+        <v>183017</v>
       </c>
       <c r="C22" t="str">
-        <v>KODIRON</v>
+        <v>SAMYONO</v>
       </c>
       <c r="D22" t="str">
-        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
+        <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E22" t="str">
-        <v>SMPN 216 KECAMATAN SENEN</v>
+        <v>SMKN 3 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F22" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G22" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H22" t="str">
-        <v>3784960</v>
+        <v>3775147</v>
       </c>
       <c r="I22">
         <v>1</v>
@@ -1108,25 +1108,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B23" t="str">
-        <v>183017</v>
+        <v>165394</v>
       </c>
       <c r="C23" t="str">
-        <v>SAMYONO</v>
+        <v>ERWIN VICTOR PARULIAN</v>
       </c>
       <c r="D23" t="str">
         <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E23" t="str">
-        <v>SMKN 3 KECAMATAN KEMAYORAN</v>
+        <v>SMKN 39 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F23" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G23" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H23" t="str">
-        <v>3775147</v>
+        <v>3770291</v>
       </c>
       <c r="I23">
         <v>1</v>
@@ -1140,25 +1140,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B24" t="str">
-        <v>186021</v>
+        <v>186336</v>
       </c>
       <c r="C24" t="str">
-        <v>EDY SARWOKO</v>
+        <v>TURMUDI</v>
       </c>
       <c r="D24" t="str">
-        <v>KEPALA SUBBAGIAN TATA USAHA</v>
+        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
       </c>
       <c r="E24" t="str">
-        <v>SMKN 31 KECAMATAN JOHAR BARU</v>
+        <v>SMPN 77 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F24" t="str">
-        <v>Draft</v>
+        <v>Penilaian akhir atas keberatan</v>
       </c>
       <c r="G24" t="str">
-        <v>Draft</v>
+        <v>Penilaian akhir atas keberatan</v>
       </c>
       <c r="H24" t="str">
-        <v>3767087</v>
+        <v>3766503</v>
       </c>
       <c r="I24">
         <v>1</v>
@@ -1172,25 +1172,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B25" t="str">
-        <v>188772</v>
+        <v>173346</v>
       </c>
       <c r="C25" t="str">
-        <v>SUTARNO</v>
+        <v>RISKY AMELIA</v>
       </c>
       <c r="D25" t="str">
         <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E25" t="str">
-        <v>SMPN 28 KECAMATAN JOHAR BARU</v>
+        <v>SMPN 47 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F25" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G25" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H25" t="str">
-        <v>3764714</v>
+        <v>3767707</v>
       </c>
       <c r="I25">
         <v>1</v>
@@ -1204,25 +1204,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B26" t="str">
-        <v>186336</v>
+        <v>222657</v>
       </c>
       <c r="C26" t="str">
-        <v>TURMUDI</v>
+        <v>MUHAMMAD NADHIRSYAH INDRA</v>
       </c>
       <c r="D26" t="str">
-        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
+        <v>STAF</v>
       </c>
       <c r="E26" t="str">
-        <v>SMPN 77 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SDN JOHAR BARU 03</v>
       </c>
       <c r="F26" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G26" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H26" t="str">
-        <v>3766503</v>
+        <v>3779978</v>
       </c>
       <c r="I26">
         <v>1</v>
@@ -1236,25 +1236,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B27" t="str">
-        <v>188455</v>
+        <v>222664</v>
       </c>
       <c r="C27" t="str">
-        <v>YULI KUSDIARTI</v>
+        <v>ILHAM ALBASITH</v>
       </c>
       <c r="D27" t="str">
-        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
+        <v>STAF</v>
       </c>
       <c r="E27" t="str">
-        <v>SMPN 10 KECAMATAN KEMAYORAN</v>
+        <v>SDN TANAH TINGGI 01</v>
       </c>
       <c r="F27" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G27" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H27" t="str">
-        <v>3783007</v>
+        <v>3762420</v>
       </c>
       <c r="I27">
         <v>1</v>
@@ -1268,10 +1268,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B28" t="str">
-        <v>222220</v>
+        <v>222216</v>
       </c>
       <c r="C28" t="str">
-        <v>SHAFIRA SHAFA RAMADHINA</v>
+        <v>DESI RATNA SARI MARIA</v>
       </c>
       <c r="D28" t="str">
         <v>STAF</v>
@@ -1280,13 +1280,13 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F28" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G28" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H28" t="str">
-        <v>3772999</v>
+        <v>3761422</v>
       </c>
       <c r="I28">
         <v>1</v>
@@ -1300,25 +1300,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B29" t="str">
-        <v>222210</v>
+        <v>182677</v>
       </c>
       <c r="C29" t="str">
-        <v>MUHAMAD ALFARISI</v>
+        <v>R.M. NURUL ZAMAN</v>
       </c>
       <c r="D29" t="str">
-        <v>STAF</v>
+        <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E29" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SMAN 27 KECAMATAN JOHAR BARU</v>
       </c>
       <c r="F29" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G29" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H29" t="str">
-        <v>3770283</v>
+        <v>3772507</v>
       </c>
       <c r="I29">
         <v>1</v>
@@ -1332,25 +1332,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B30" t="str">
-        <v>223987</v>
+        <v>189725</v>
       </c>
       <c r="C30" t="str">
-        <v>DESTI RAHMAWATI</v>
+        <v>HERYADI</v>
       </c>
       <c r="D30" t="str">
-        <v>STAF</v>
+        <v>STAF PELAYANAN TINGKAT TERAMPIL</v>
       </c>
       <c r="E30" t="str">
-        <v>SDN JOHAR BARU 13</v>
+        <v>SDN PASEBAN 15 PAGI</v>
       </c>
       <c r="F30" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G30" t="str">
-        <v>Belum Ada</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H30" t="str">
-        <v>3764661</v>
+        <v>3762438</v>
       </c>
       <c r="I30">
         <v>1</v>
@@ -1364,25 +1364,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B31" t="str">
-        <v>135533</v>
+        <v>163673</v>
       </c>
       <c r="C31" t="str">
-        <v>ENDANG RAHAYU NINGSIH</v>
+        <v>SEMIATI</v>
       </c>
       <c r="D31" t="str">
-        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
+        <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E31" t="str">
-        <v>SMPN 137 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SMAN 30 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F31" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G31" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H31" t="str">
-        <v>3767188</v>
+        <v>3765532</v>
       </c>
       <c r="I31">
         <v>1</v>
@@ -1396,25 +1396,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B32" t="str">
-        <v>212701</v>
+        <v>222662</v>
       </c>
       <c r="C32" t="str">
-        <v>INA NURNINA</v>
+        <v>DAFFA AL HAFIZH</v>
       </c>
       <c r="D32" t="str">
-        <v>KEPALA SUBBAGIAN TATA USAHA</v>
+        <v>STAF</v>
       </c>
       <c r="E32" t="str">
-        <v>SMKN 54 KECAMATAN KEMAYORAN</v>
+        <v>SDN JOHAR BARU 15</v>
       </c>
       <c r="F32" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G32" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H32" t="str">
-        <v>3772702</v>
+        <v>3784660</v>
       </c>
       <c r="I32">
         <v>1</v>
@@ -1428,25 +1428,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B33" t="str">
-        <v>222660</v>
+        <v>133473</v>
       </c>
       <c r="C33" t="str">
-        <v>VEGA PUTRA PRADANA</v>
+        <v>SITI RAMROH</v>
       </c>
       <c r="D33" t="str">
-        <v>STAF</v>
+        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
       </c>
       <c r="E33" t="str">
-        <v>SDN JOHAR BARU 09 PAGI</v>
+        <v>SMPN 71 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F33" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G33" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H33" t="str">
-        <v>3775885</v>
+        <v>3771906</v>
       </c>
       <c r="I33">
         <v>1</v>
@@ -1460,25 +1460,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B34" t="str">
-        <v>222665</v>
+        <v>222667</v>
       </c>
       <c r="C34" t="str">
-        <v>DIPA ANGGRIAWAN</v>
+        <v>MOCH. SANDI ALPANSURI</v>
       </c>
       <c r="D34" t="str">
         <v>STAF</v>
       </c>
       <c r="E34" t="str">
-        <v>SDN TANAH TINGGI 03</v>
+        <v>SDN TANAH TINGGI 09</v>
       </c>
       <c r="F34" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G34" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H34" t="str">
-        <v>3781183</v>
+        <v>3766228</v>
       </c>
       <c r="I34">
         <v>1</v>
@@ -1492,25 +1492,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B35" t="str">
-        <v>143266</v>
+        <v>188455</v>
       </c>
       <c r="C35" t="str">
-        <v>SUTARNO</v>
+        <v>YULI KUSDIARTI</v>
       </c>
       <c r="D35" t="str">
-        <v>KEPALA SUBBAGIAN TATA USAHA</v>
+        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
       </c>
       <c r="E35" t="str">
-        <v>SMAN 77 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SMPN 10 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F35" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G35" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H35" t="str">
-        <v>3768510</v>
+        <v>3783007</v>
       </c>
       <c r="I35">
         <v>1</v>
@@ -1524,25 +1524,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B36" t="str">
-        <v>222664</v>
+        <v>222647</v>
       </c>
       <c r="C36" t="str">
-        <v>ILHAM ALBASITH</v>
+        <v>GHINA KAMILAH</v>
       </c>
       <c r="D36" t="str">
         <v>STAF</v>
       </c>
       <c r="E36" t="str">
-        <v>SDN TANAH TINGGI 01</v>
+        <v>SDN SUMUR BATU 08</v>
       </c>
       <c r="F36" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G36" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H36" t="str">
-        <v>3762420</v>
+        <v>3782730</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -1556,25 +1556,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B37" t="str">
-        <v>222207</v>
+        <v>176997</v>
       </c>
       <c r="C37" t="str">
-        <v>YAN AJIE PRASETIA</v>
+        <v>YENDHA PUTRI WULANDARI</v>
       </c>
       <c r="D37" t="str">
-        <v>STAF</v>
+        <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E37" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SMKN 14 KECAMATAN JOHAR BARU</v>
       </c>
       <c r="F37" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G37" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H37" t="str">
-        <v>3762888</v>
+        <v>3762685</v>
       </c>
       <c r="I37">
         <v>1</v>
@@ -1588,10 +1588,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B38" t="str">
-        <v>222224</v>
+        <v>222218</v>
       </c>
       <c r="C38" t="str">
-        <v>IHSAN MAULANA ILMI</v>
+        <v>NIRWANA PRATIWI</v>
       </c>
       <c r="D38" t="str">
         <v>STAF</v>
@@ -1600,13 +1600,13 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F38" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G38" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H38" t="str">
-        <v>3762076</v>
+        <v>3785348</v>
       </c>
       <c r="I38">
         <v>1</v>
@@ -1620,10 +1620,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B39" t="str">
-        <v>222213</v>
+        <v>222220</v>
       </c>
       <c r="C39" t="str">
-        <v>FEBBY FEBRIANA</v>
+        <v>SHAFIRA SHAFA RAMADHINA</v>
       </c>
       <c r="D39" t="str">
         <v>STAF</v>
@@ -1632,13 +1632,13 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F39" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G39" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H39" t="str">
-        <v>3765037</v>
+        <v>3772999</v>
       </c>
       <c r="I39">
         <v>1</v>
@@ -1652,10 +1652,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B40" t="str">
-        <v>222222</v>
+        <v>222214</v>
       </c>
       <c r="C40" t="str">
-        <v>KRISNA PRAMULYA PUTRA</v>
+        <v>SALMAN AFFANDI</v>
       </c>
       <c r="D40" t="str">
         <v>STAF</v>
@@ -1664,13 +1664,13 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F40" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G40" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H40" t="str">
-        <v>3774731</v>
+        <v>3783118</v>
       </c>
       <c r="I40">
         <v>1</v>
@@ -1696,10 +1696,10 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F41" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G41" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H41" t="str">
         <v>3781386</v>
@@ -1716,25 +1716,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B42" t="str">
-        <v>172324</v>
+        <v>185754</v>
       </c>
       <c r="C42" t="str">
-        <v>RIZA MARDIANA WARDHANI</v>
+        <v>KODIRON</v>
       </c>
       <c r="D42" t="str">
-        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
+        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
       </c>
       <c r="E42" t="str">
-        <v>SMPN 119 KECAMATAN KEMAYORAN</v>
+        <v>SMPN 216 KECAMATAN SENEN</v>
       </c>
       <c r="F42" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G42" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H42" t="str">
-        <v>3768052</v>
+        <v>3784960</v>
       </c>
       <c r="I42">
         <v>1</v>
@@ -1748,25 +1748,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B43" t="str">
-        <v>191415</v>
+        <v>172324</v>
       </c>
       <c r="C43" t="str">
-        <v>RIKA MULYANINGSIH</v>
+        <v>RIZA MARDIANA WARDHANI</v>
       </c>
       <c r="D43" t="str">
         <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E43" t="str">
-        <v>SMPN 78 KECAMATAN KEMAYORAN</v>
+        <v>SMPN 119 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F43" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G43" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H43" t="str">
-        <v>3766529</v>
+        <v>3768052</v>
       </c>
       <c r="I43">
         <v>1</v>
@@ -1780,25 +1780,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B44" t="str">
-        <v>222667</v>
+        <v>222658</v>
       </c>
       <c r="C44" t="str">
-        <v>MOCH. SANDI ALPANSURI</v>
+        <v>MUHAMAD NUR RIDWAN</v>
       </c>
       <c r="D44" t="str">
         <v>STAF</v>
       </c>
       <c r="E44" t="str">
-        <v>SDN TANAH TINGGI 09</v>
+        <v>SDN JOHAR BARU 04</v>
       </c>
       <c r="F44" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G44" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H44" t="str">
-        <v>3766228</v>
+        <v>3781889</v>
       </c>
       <c r="I44">
         <v>1</v>
@@ -1812,25 +1812,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B45" t="str">
-        <v>164920</v>
+        <v>143266</v>
       </c>
       <c r="C45" t="str">
-        <v>SYARIF YUSUF</v>
+        <v>SUTARNO</v>
       </c>
       <c r="D45" t="str">
         <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E45" t="str">
-        <v>SMKN 34 KECAMATAN SENEN</v>
+        <v>SMAN 77 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F45" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G45" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H45" t="str">
-        <v>3769210</v>
+        <v>3768510</v>
       </c>
       <c r="I45">
         <v>1</v>
@@ -1844,25 +1844,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B46" t="str">
-        <v>222646</v>
+        <v>189627</v>
       </c>
       <c r="C46" t="str">
-        <v>RETNO WULANDARI</v>
+        <v>SUMANTO WIRYAWAN</v>
       </c>
       <c r="D46" t="str">
-        <v>STAF</v>
+        <v>STAF TEKNIS TINGKAT AHLI</v>
       </c>
       <c r="E46" t="str">
-        <v>SDN HARAPAN MULIA 03</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F46" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G46" t="str">
-        <v>Belum Ada</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H46" t="str">
-        <v>3765436</v>
+        <v>3786263</v>
       </c>
       <c r="I46">
         <v>1</v>
@@ -1876,25 +1876,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B47" t="str">
-        <v>171594</v>
+        <v>222212</v>
       </c>
       <c r="C47" t="str">
-        <v>SAFITRI HARUN</v>
+        <v>ERICK LAUSHEN</v>
       </c>
       <c r="D47" t="str">
-        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
+        <v>STAF</v>
       </c>
       <c r="E47" t="str">
-        <v>SMPN 118 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F47" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G47" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H47" t="str">
-        <v>3763657</v>
+        <v>3764322</v>
       </c>
       <c r="I47">
         <v>1</v>
@@ -1908,10 +1908,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B48" t="str">
-        <v>222223</v>
+        <v>222206</v>
       </c>
       <c r="C48" t="str">
-        <v>MUHAMMAD ZUFAR GIFFARY</v>
+        <v>FARIZ SEPTIAN</v>
       </c>
       <c r="D48" t="str">
         <v>STAF</v>
@@ -1920,13 +1920,13 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F48" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G48" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H48" t="str">
-        <v>3766960</v>
+        <v>3771045</v>
       </c>
       <c r="I48">
         <v>1</v>
@@ -1940,25 +1940,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B49" t="str">
-        <v>197054</v>
+        <v>186567</v>
       </c>
       <c r="C49" t="str">
-        <v>ANDRIE GUSTYAJI</v>
+        <v>DAHIYAT</v>
       </c>
       <c r="D49" t="str">
-        <v>STAF TEKNIS TINGKAT AHLI</v>
+        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
       </c>
       <c r="E49" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SMPN 137 KECAMATAN CEMPAKA PUTIH</v>
       </c>
       <c r="F49" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G49" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H49" t="str">
-        <v>3767464</v>
+        <v>3784901</v>
       </c>
       <c r="I49">
         <v>1</v>
@@ -1972,25 +1972,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B50" t="str">
-        <v>222214</v>
+        <v>141357</v>
       </c>
       <c r="C50" t="str">
-        <v>SALMAN AFFANDI</v>
+        <v>HERI BUDI PRASETYA</v>
       </c>
       <c r="D50" t="str">
-        <v>STAF</v>
+        <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E50" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SMAN 68 KECAMATAN SENEN</v>
       </c>
       <c r="F50" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G50" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H50" t="str">
-        <v>3783118</v>
+        <v>3771889</v>
       </c>
       <c r="I50">
         <v>1</v>
@@ -2004,25 +2004,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B51" t="str">
-        <v>189627</v>
+        <v>212701</v>
       </c>
       <c r="C51" t="str">
-        <v>SUMANTO WIRYAWAN</v>
+        <v>INA NURNINA</v>
       </c>
       <c r="D51" t="str">
-        <v>STAF TEKNIS TINGKAT AHLI</v>
+        <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E51" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SMKN 54 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F51" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G51" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H51" t="str">
-        <v>3786263</v>
+        <v>3772702</v>
       </c>
       <c r="I51">
         <v>1</v>
@@ -2036,25 +2036,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B52" t="str">
-        <v>186932</v>
+        <v>222665</v>
       </c>
       <c r="C52" t="str">
-        <v>VINSKA PUSPITA</v>
+        <v>DIPA ANGGRIAWAN</v>
       </c>
       <c r="D52" t="str">
-        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
+        <v>STAF</v>
       </c>
       <c r="E52" t="str">
-        <v>SMPN 216 KECAMATAN SENEN</v>
+        <v>SDN TANAH TINGGI 03</v>
       </c>
       <c r="F52" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G52" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H52" t="str">
-        <v>3773561</v>
+        <v>3781183</v>
       </c>
       <c r="I52">
         <v>1</v>
@@ -2068,25 +2068,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B53" t="str">
-        <v>121949</v>
+        <v>222663</v>
       </c>
       <c r="C53" t="str">
-        <v>RIA SCORPIONI</v>
+        <v>ZAINAL NUR ROKIB</v>
       </c>
       <c r="D53" t="str">
-        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
+        <v>STAF</v>
       </c>
       <c r="E53" t="str">
-        <v>SMPN 79 KECAMATAN KEMAYORAN</v>
+        <v>SDN JOHAR BARU 17</v>
       </c>
       <c r="F53" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G53" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H53" t="str">
-        <v>3784557</v>
+        <v>3783748</v>
       </c>
       <c r="I53">
         <v>1</v>
@@ -2100,25 +2100,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B54" t="str">
-        <v>222658</v>
+        <v>222221</v>
       </c>
       <c r="C54" t="str">
-        <v>MUHAMAD NUR RIDWAN</v>
+        <v>TASKIA ROROINTAN SUGYANTI</v>
       </c>
       <c r="D54" t="str">
         <v>STAF</v>
       </c>
       <c r="E54" t="str">
-        <v>SDN JOHAR BARU 04</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F54" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G54" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H54" t="str">
-        <v>3781889</v>
+        <v>3775540</v>
       </c>
       <c r="I54">
         <v>1</v>
@@ -2132,25 +2132,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B55" t="str">
-        <v>182690</v>
+        <v>222215</v>
       </c>
       <c r="C55" t="str">
-        <v>SALYA</v>
+        <v>ABIYU MUHAMMAD AKMAL</v>
       </c>
       <c r="D55" t="str">
-        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
+        <v>STAF</v>
       </c>
       <c r="E55" t="str">
-        <v>SMPN 71 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F55" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G55" t="str">
-        <v>Draft</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H55" t="str">
-        <v>3766145</v>
+        <v>3769250</v>
       </c>
       <c r="I55">
         <v>1</v>
@@ -2164,25 +2164,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B56" t="str">
-        <v>222647</v>
+        <v>222648</v>
       </c>
       <c r="C56" t="str">
-        <v>GHINA KAMILAH</v>
+        <v>ZOEL ROCHMAN BUDJANA</v>
       </c>
       <c r="D56" t="str">
         <v>STAF</v>
       </c>
       <c r="E56" t="str">
-        <v>SDN SUMUR BATU 08</v>
+        <v>SDN SUMUR BATU 12 PAGI</v>
       </c>
       <c r="F56" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G56" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H56" t="str">
-        <v>3782730</v>
+        <v>3767061</v>
       </c>
       <c r="I56">
         <v>1</v>
@@ -2196,25 +2196,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B57" t="str">
-        <v>121745</v>
+        <v>142108</v>
       </c>
       <c r="C57" t="str">
-        <v>ROSDIANA</v>
+        <v>SADONO</v>
       </c>
       <c r="D57" t="str">
         <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E57" t="str">
-        <v>SMKN 44 KECAMATAN KEMAYORAN</v>
+        <v>SMKN 21 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F57" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G57" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H57" t="str">
-        <v>3772076</v>
+        <v>3763827</v>
       </c>
       <c r="I57">
         <v>1</v>
@@ -2228,25 +2228,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B58" t="str">
-        <v>137905</v>
+        <v>117752</v>
       </c>
       <c r="C58" t="str">
-        <v>MELIA</v>
+        <v>IMAM SUSANTO</v>
       </c>
       <c r="D58" t="str">
-        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
+        <v>STAF PELAYANAN TINGKAT AHLI</v>
       </c>
       <c r="E58" t="str">
-        <v>SMPN 76 KECAMATAN JOHAR BARU</v>
+        <v>SDN SERDANG 05 PAGI</v>
       </c>
       <c r="F58" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G58" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H58" t="str">
-        <v>3764712</v>
+        <v>3761754</v>
       </c>
       <c r="I58">
         <v>1</v>
@@ -2260,25 +2260,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B59" t="str">
-        <v>142108</v>
+        <v>222213</v>
       </c>
       <c r="C59" t="str">
-        <v>SADONO</v>
+        <v>FEBBY FEBRIANA</v>
       </c>
       <c r="D59" t="str">
-        <v>KEPALA SUBBAGIAN TATA USAHA</v>
+        <v>STAF</v>
       </c>
       <c r="E59" t="str">
-        <v>SMKN 21 KECAMATAN KEMAYORAN</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F59" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G59" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H59" t="str">
-        <v>3763827</v>
+        <v>3765037</v>
       </c>
       <c r="I59">
         <v>1</v>
@@ -2292,25 +2292,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B60" t="str">
-        <v>222659</v>
+        <v>222649</v>
       </c>
       <c r="C60" t="str">
-        <v>RIZKI PORMAN SIDABUTAR</v>
+        <v>AHMAD SUPRIYANTO</v>
       </c>
       <c r="D60" t="str">
         <v>STAF</v>
       </c>
       <c r="E60" t="str">
-        <v>SDN JOHAR BARU 07 PAGI</v>
+        <v>SDN SUMUR BATU 14</v>
       </c>
       <c r="F60" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G60" t="str">
-        <v>Belum Ada</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H60" t="str">
-        <v>3785646</v>
+        <v>3775544</v>
       </c>
       <c r="I60">
         <v>1</v>
@@ -2324,25 +2324,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B61" t="str">
-        <v>186620</v>
+        <v>171293</v>
       </c>
       <c r="C61" t="str">
-        <v>ENDANG ERWIN</v>
+        <v>DEVIA ROSA</v>
       </c>
       <c r="D61" t="str">
-        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
+        <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E61" t="str">
-        <v>SMPN 118 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SMAN 5 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F61" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G61" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H61" t="str">
-        <v>3767642</v>
+        <v>3762691</v>
       </c>
       <c r="I61">
         <v>1</v>
@@ -2356,25 +2356,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B62" t="str">
-        <v>176997</v>
+        <v>164920</v>
       </c>
       <c r="C62" t="str">
-        <v>YENDHA PUTRI WULANDARI</v>
+        <v>SYARIF YUSUF</v>
       </c>
       <c r="D62" t="str">
         <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E62" t="str">
-        <v>SMKN 14 KECAMATAN JOHAR BARU</v>
+        <v>SMKN 34 KECAMATAN SENEN</v>
       </c>
       <c r="F62" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G62" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H62" t="str">
-        <v>3762685</v>
+        <v>3769210</v>
       </c>
       <c r="I62">
         <v>1</v>
@@ -2388,25 +2388,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B63" t="str">
-        <v>222645</v>
+        <v>222217</v>
       </c>
       <c r="C63" t="str">
-        <v>MEGANANDA DWI FITRIYANI</v>
+        <v>MUHAMMAD IHSAN</v>
       </c>
       <c r="D63" t="str">
         <v>STAF</v>
       </c>
       <c r="E63" t="str">
-        <v>SDN HARAPAN MULIA 01</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F63" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G63" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H63" t="str">
-        <v>3783067</v>
+        <v>3766043</v>
       </c>
       <c r="I63">
         <v>1</v>
@@ -2420,25 +2420,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B64" t="str">
-        <v>222666</v>
+        <v>222223</v>
       </c>
       <c r="C64" t="str">
-        <v>SYAFRIZAL</v>
+        <v>MUHAMMAD ZUFAR GIFFARY</v>
       </c>
       <c r="D64" t="str">
         <v>STAF</v>
       </c>
       <c r="E64" t="str">
-        <v>SDN TANAH TINGGI 05</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F64" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G64" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H64" t="str">
-        <v>3769614</v>
+        <v>3766960</v>
       </c>
       <c r="I64">
         <v>1</v>
@@ -2452,25 +2452,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B65" t="str">
-        <v>117752</v>
+        <v>222208</v>
       </c>
       <c r="C65" t="str">
-        <v>IMAM SUSANTO</v>
+        <v>KUNTI DEWI AFIFA</v>
       </c>
       <c r="D65" t="str">
-        <v>STAF PELAYANAN TINGKAT AHLI</v>
+        <v>STAF</v>
       </c>
       <c r="E65" t="str">
-        <v>SDN SERDANG 05 PAGI</v>
+        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F65" t="str">
-        <v>Persetujuan pegawai</v>
+        <v>Selesai</v>
       </c>
       <c r="G65" t="str">
-        <v>Persetujuan pegawai</v>
+        <v>Baik</v>
       </c>
       <c r="H65" t="str">
-        <v>3761754</v>
+        <v>3773218</v>
       </c>
       <c r="I65">
         <v>1</v>
@@ -2484,10 +2484,10 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B66" t="str">
-        <v>222217</v>
+        <v>222222</v>
       </c>
       <c r="C66" t="str">
-        <v>MUHAMMAD IHSAN</v>
+        <v>KRISNA PRAMULYA PUTRA</v>
       </c>
       <c r="D66" t="str">
         <v>STAF</v>
@@ -2496,13 +2496,13 @@
         <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
       </c>
       <c r="F66" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G66" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H66" t="str">
-        <v>3766043</v>
+        <v>3774731</v>
       </c>
       <c r="I66">
         <v>1</v>
@@ -2516,25 +2516,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B67" t="str">
-        <v>222215</v>
+        <v>186932</v>
       </c>
       <c r="C67" t="str">
-        <v>ABIYU MUHAMMAD AKMAL</v>
+        <v>VINSKA PUSPITA</v>
       </c>
       <c r="D67" t="str">
-        <v>STAF</v>
+        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E67" t="str">
-        <v>SUKU DINAS PENDIDIKAN WILAYAH II KOTA ADM. JAKARTA PUSAT</v>
+        <v>SMPN 216 KECAMATAN SENEN</v>
       </c>
       <c r="F67" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G67" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H67" t="str">
-        <v>3769250</v>
+        <v>3773561</v>
       </c>
       <c r="I67">
         <v>1</v>
@@ -2560,10 +2560,10 @@
         <v>SMPN 2 KECAMATAN JOHAR BARU</v>
       </c>
       <c r="F68" t="str">
-        <v>Persetujuan pegawai</v>
+        <v>Selesai</v>
       </c>
       <c r="G68" t="str">
-        <v>Persetujuan pegawai</v>
+        <v>Baik</v>
       </c>
       <c r="H68" t="str">
         <v>3762732</v>
@@ -2580,25 +2580,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B69" t="str">
-        <v>222656</v>
+        <v>223987</v>
       </c>
       <c r="C69" t="str">
-        <v>HANDY WICAKSONO</v>
+        <v>DESTI RAHMAWATI</v>
       </c>
       <c r="D69" t="str">
         <v>STAF</v>
       </c>
       <c r="E69" t="str">
-        <v>SDN JOHAR BARU 01 PAGI</v>
+        <v>SDN JOHAR BARU 13</v>
       </c>
       <c r="F69" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="G69" t="str">
-        <v>Belum Ada</v>
+        <v>Persetujuan pegawai</v>
       </c>
       <c r="H69" t="str">
-        <v>3783616</v>
+        <v>3764661</v>
       </c>
       <c r="I69">
         <v>1</v>
@@ -2612,25 +2612,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B70" t="str">
-        <v>222648</v>
+        <v>121745</v>
       </c>
       <c r="C70" t="str">
-        <v>ZOEL ROCHMAN BUDJANA</v>
+        <v>ROSDIANA</v>
       </c>
       <c r="D70" t="str">
-        <v>STAF</v>
+        <v>KEPALA SUBBAGIAN TATA USAHA</v>
       </c>
       <c r="E70" t="str">
-        <v>SDN SUMUR BATU 12 PAGI</v>
+        <v>SMKN 44 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F70" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G70" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H70" t="str">
-        <v>3767061</v>
+        <v>3772076</v>
       </c>
       <c r="I70">
         <v>1</v>
@@ -2656,10 +2656,10 @@
         <v>SMPN 269 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F71" t="str">
-        <v>Persetujuan pegawai</v>
+        <v>Selesai</v>
       </c>
       <c r="G71" t="str">
-        <v>Persetujuan pegawai</v>
+        <v>Baik</v>
       </c>
       <c r="H71" t="str">
         <v>3766911</v>
@@ -2676,25 +2676,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B72" t="str">
-        <v>222662</v>
+        <v>222660</v>
       </c>
       <c r="C72" t="str">
-        <v>DAFFA AL HAFIZH</v>
+        <v>VEGA PUTRA PRADANA</v>
       </c>
       <c r="D72" t="str">
         <v>STAF</v>
       </c>
       <c r="E72" t="str">
-        <v>SDN JOHAR BARU 15</v>
+        <v>SDN JOHAR BARU 09 PAGI</v>
       </c>
       <c r="F72" t="str">
-        <v>Verifikasi pejabat penilai</v>
+        <v>Selesai</v>
       </c>
       <c r="G72" t="str">
-        <v>Belum Ada</v>
+        <v>Baik</v>
       </c>
       <c r="H72" t="str">
-        <v>3784660</v>
+        <v>3775885</v>
       </c>
       <c r="I72">
         <v>1</v>
@@ -2708,25 +2708,25 @@
         <v>Bawahan Tidak Langsung</v>
       </c>
       <c r="B73" t="str">
-        <v>133473</v>
+        <v>191415</v>
       </c>
       <c r="C73" t="str">
-        <v>SITI RAMROH</v>
+        <v>RIKA MULYANINGSIH</v>
       </c>
       <c r="D73" t="str">
-        <v>STAF ADMINISTRASI TINGKAT TERAMPIL</v>
+        <v>KEPALA SATUAN PELAKSANA TATA USAHA SMP</v>
       </c>
       <c r="E73" t="str">
-        <v>SMPN 71 KECAMATAN CEMPAKA PUTIH</v>
+        <v>SMPN 78 KECAMATAN KEMAYORAN</v>
       </c>
       <c r="F73" t="str">
-        <v>Draft</v>
+        <v>Selesai</v>
       </c>
       <c r="G73" t="str">
-        <v>Draft</v>
+        <v>Baik</v>
       </c>
       <c r="H73" t="str">
-        <v>3771906</v>
+        <v>3766529</v>
       </c>
       <c r="I73">
         <v>1</v>

</xml_diff>